<commit_message>
fix(skills): correct glyph token-cost claim; drop cross-variant @ from classical fixture
</commit_message>
<xml_diff>
--- a/test/results/token-savings.xlsx
+++ b/test/results/token-savings.xlsx
@@ -588,7 +588,7 @@
         <v>30</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>405</v>
+        <v>703</v>
       </c>
     </row>
     <row r="5">
@@ -1268,7 +1268,7 @@
       <c r="A1" s="5" t="inlineStr">
         <is>
           <t>{
-  "measuredAt": "2026-05-13T19:00:56.268Z",
+  "measuredAt": "2026-05-14T02:01:34.227Z",
   "tokenizer": "cl100k_base",
   "methodology": "Baseline output tokens are a constant 120 placeholder (typical verbose reply). Real Claude-reply measurements deferred to FUTURE_WORK.md. Tokenizer is js-tiktoken cl100k_base — NOT Anthropic's tokenizer, so absolute counts are directional only.",
   "variants": [
@@ -1296,7 +1296,7 @@
           "savingsPct": 72.5
         },
         "tc-mirror-glyphs": {
-          "skillOverheadTokens": 405,
+          "skillOverheadTokens": 703,
           "expectedOutputTokens": 30,
           "savingsPct": 75
         },
@@ -1325,7 +1325,7 @@
           "savingsPct": null
         },
         "tc-mirror-glyphs": {
-          "skillOverheadTokens": 405,
+          "skillOverheadTokens": 703,
           "expectedOutputTokens": null,
           "savingsPct": null
         },
@@ -1354,7 +1354,7 @@
           "savingsPct": null
         },
         "tc-mirror-glyphs": {
-          "skillOverheadTokens": 405,
+          "skillOverheadTokens": 703,
           "expectedOutputTokens": null,
           "savingsPct": null
         },
@@ -1383,7 +1383,7 @@
           "savingsPct": null
         },
         "tc-mirror-glyphs": {
-          "skillOverheadTokens": 405,
+          "skillOverheadTokens": 703,
           "expectedOutputTokens": null,
           "savingsPct": null
         },
@@ -1412,7 +1412,7 @@
           "savingsPct": null
         },
         "tc-mirror-glyphs": {
-          "skillOverheadTokens": 405,
+          "skillOverheadTokens": 703,
           "expectedOutputTokens": null,
           "savingsPct": null
         },
@@ -1441,7 +1441,7 @@
           "savingsPct": null
         },
         "tc-mirror-glyphs": {
-          "skillOverheadTokens": 405,
+          "skillOverheadTokens": 703,
           "expectedOutputTokens": null,
           "savingsPct": null
         },
@@ -1470,7 +1470,7 @@
           "savingsPct": null
         },
         "tc-mirror-glyphs": {
-          "skillOverheadTokens": 405,
+          "skillOverheadTokens": 703,
           "expectedOutputTokens": null,
           "savingsPct": null
         },
@@ -1499,7 +1499,7 @@
           "savingsPct": null
         },
         "tc-mirror-glyphs": {
-          "skillOverheadTokens": 405,
+          "skillOverheadTokens": 703,
           "expectedOutputTokens": null,
           "savingsPct": null
         },
@@ -1601,7 +1601,7 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>2026-05-13T19:00:56.268Z</t>
+          <t>2026-05-14T02:01:34.227Z</t>
         </is>
       </c>
     </row>

</xml_diff>